<commit_message>
feat: club radar and builder directory, add city center distance benchmark, property age vs completion matrix, and dynamic budget refresh
</commit_message>
<xml_diff>
--- a/data/daily_property_screener_dump.xlsx
+++ b/data/daily_property_screener_dump.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z11"/>
+  <dimension ref="A1:AA19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -478,75 +478,80 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>Property Age vs Completion Timeline</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>Upcoming Phase</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Configuration</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Avg Sqft</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Price / Sqft (INR)</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Total Price (Cr)</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Plinth Elevation (m MSL)</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Flood Risk Category</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>STP Setup</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Water Softener</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>IoT Water Meter</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Piped Gas</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Investment Score (0-100)</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Critic AI Status</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>Primary RERA Link</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>Data Source Verification</t>
         </is>
@@ -560,7 +565,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -610,65 +615,70 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
+          <t>🏗️ Under Construction (Dec 2026 • 14 mos)</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
           <t>Tower 4 &amp; 5 (Structure Complete)</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>3 BHK Luxury</t>
         </is>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>1820</v>
       </c>
-      <c r="O2" t="n">
+      <c r="P2" t="n">
         <v>14200</v>
       </c>
-      <c r="P2" t="n">
+      <c r="Q2" t="n">
         <v>2.58</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="R2" t="n">
         <v>884</v>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>High Plinth (Elevated Natural Ridge)</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>MBBR Biological STP</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="W2" t="n">
+      <c r="X2" t="n">
         <v>94.8</v>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t>✅ Critic AI Validated</t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="Z2" t="inlineStr">
         <is>
           <t>https://rera.karnataka.gov.in/</t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AA2" t="inlineStr">
         <is>
           <t>State RERA Registry (Sobha Limited Legal Filing) | Municipal Stormwater Master Plan (GIS Contour Elevation) | TomTom / Google Mobility Commute Index | Public Works Department / Metro Phase Infrastructure Blueprint</t>
         </is>
@@ -682,7 +692,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -732,65 +742,70 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
+          <t>🟢 Ready to Move (4 yrs old • Active Community)</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
           <t>Completed Phase with Occupancy Certificate</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>3 BHK Premium</t>
         </is>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>1780</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>12800</v>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>2.28</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>912</v>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>Zero Inundation (High Table-land)</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>MBBR Biological STP</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="W3" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="W3" t="n">
+      <c r="X3" t="n">
         <v>93.2</v>
       </c>
-      <c r="X3" t="inlineStr">
+      <c r="Y3" t="inlineStr">
         <is>
           <t>✅ Critic AI Validated</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
+      <c r="Z3" t="inlineStr">
         <is>
           <t>https://rera.karnataka.gov.in/</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="AA3" t="inlineStr">
         <is>
           <t>State RERA Registry (Prestige Group Legal Filing) | Municipal Stormwater Master Plan (GIS Contour Elevation) | TomTom / Google Mobility Commute Index | Public Works Department / Metro Phase Infrastructure Blueprint</t>
         </is>
@@ -804,7 +819,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -854,65 +869,70 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
+          <t>🚀 Upcoming Pre-Launch (March 2027 • ~2 yrs)</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
           <t>Phase 2 Wing C (Foundation in Progress)</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>3 BHK Smart Luxury</t>
         </is>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>1640</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>11900</v>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
         <v>1.95</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="R4" t="n">
         <v>885</v>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>Engineered SWD with High Berm Buffer</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>MBBR Biological STP</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="W4" t="n">
+      <c r="X4" t="n">
         <v>92.40000000000001</v>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>✅ Critic AI Validated</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>https://rera.karnataka.gov.in/</t>
         </is>
       </c>
-      <c r="Z4" t="inlineStr">
+      <c r="AA4" t="inlineStr">
         <is>
           <t>State RERA Registry (Brigade Group Legal Filing) | Municipal Stormwater Master Plan (GIS Contour Elevation) | TomTom / Google Mobility Commute Index | Public Works Department / Metro Phase Infrastructure Blueprint</t>
         </is>
@@ -926,7 +946,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -976,65 +996,70 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
+          <t>🏗️ Under Construction (June 2026 • 8 mos)</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
           <t>Tower Horizon (Finishing Works)</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>3 BHK Grande</t>
         </is>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>1420</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>26800</v>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
         <v>3.81</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="R5" t="n">
         <v>38</v>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>Zero Inundation (Natural Granitic Base)</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>MBBR Biological STP</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="W5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="W5" t="n">
+      <c r="X5" t="n">
         <v>96.2</v>
       </c>
-      <c r="X5" t="inlineStr">
+      <c r="Y5" t="inlineStr">
         <is>
           <t>✅ Critic AI Validated</t>
         </is>
       </c>
-      <c r="Y5" t="inlineStr">
+      <c r="Z5" t="inlineStr">
         <is>
           <t>https://maharera.mahaonline.gov.in/</t>
         </is>
       </c>
-      <c r="Z5" t="inlineStr">
+      <c r="AA5" t="inlineStr">
         <is>
           <t>State RERA Registry (Oberoi Realty Legal Filing) | Municipal Stormwater Master Plan (GIS Contour Elevation) | TomTom / Google Mobility Commute Index | Public Works Department / Metro Phase Infrastructure Blueprint</t>
         </is>
@@ -1048,7 +1073,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1098,65 +1123,70 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
+          <t>🏗️ Near Completion (Dec 2025 • ~2 mos)</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
           <t>Avenue 3 (OC Expected Q4 2025)</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>3 BHK Transit-Oriented</t>
         </is>
       </c>
-      <c r="N6" t="n">
+      <c r="O6" t="n">
         <v>1350</v>
       </c>
-      <c r="O6" t="n">
+      <c r="P6" t="n">
         <v>21500</v>
       </c>
-      <c r="P6" t="n">
+      <c r="Q6" t="n">
         <v>2.9</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="R6" t="n">
         <v>12</v>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>Engineered CIDCO Polder Drainage (No waterlogging)</t>
         </is>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>MBBR Biological STP</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="V6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="V6" t="inlineStr">
+      <c r="W6" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="W6" t="n">
+      <c r="X6" t="n">
         <v>94.5</v>
       </c>
-      <c r="X6" t="inlineStr">
+      <c r="Y6" t="inlineStr">
         <is>
           <t>✅ Critic AI Validated</t>
         </is>
       </c>
-      <c r="Y6" t="inlineStr">
+      <c r="Z6" t="inlineStr">
         <is>
           <t>https://maharera.mahaonline.gov.in/</t>
         </is>
       </c>
-      <c r="Z6" t="inlineStr">
+      <c r="AA6" t="inlineStr">
         <is>
           <t>State RERA Registry (L&amp;T Realty Legal Filing) | Municipal Stormwater Master Plan (GIS Contour Elevation) | TomTom / Google Mobility Commute Index | Public Works Department / Metro Phase Infrastructure Blueprint</t>
         </is>
@@ -1170,7 +1200,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1220,65 +1250,70 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
+          <t>🏗️ Under Construction (March 2027 • 17 mos)</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
           <t>Palais Royale Wing B (Under Construction)</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>3 BHK Sustainable Suite</t>
         </is>
       </c>
-      <c r="N7" t="n">
+      <c r="O7" t="n">
         <v>1490</v>
       </c>
-      <c r="O7" t="n">
+      <c r="P7" t="n">
         <v>25500</v>
       </c>
-      <c r="P7" t="n">
+      <c r="Q7" t="n">
         <v>3.8</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="R7" t="n">
         <v>16</v>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="S7" t="inlineStr">
         <is>
           <t>Zero Inundation (Protected Mangrove Buffer Zone)</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>MBBR Biological STP</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="V7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="V7" t="inlineStr">
+      <c r="W7" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="W7" t="n">
+      <c r="X7" t="n">
         <v>93.90000000000001</v>
       </c>
-      <c r="X7" t="inlineStr">
+      <c r="Y7" t="inlineStr">
         <is>
           <t>✅ Critic AI Validated</t>
         </is>
       </c>
-      <c r="Y7" t="inlineStr">
+      <c r="Z7" t="inlineStr">
         <is>
           <t>https://maharera.mahaonline.gov.in/</t>
         </is>
       </c>
-      <c r="Z7" t="inlineStr">
+      <c r="AA7" t="inlineStr">
         <is>
           <t>State RERA Registry (Godrej Properties Legal Filing) | Municipal Stormwater Master Plan (GIS Contour Elevation) | TomTom / Google Mobility Commute Index | Public Works Department / Metro Phase Infrastructure Blueprint</t>
         </is>
@@ -1292,7 +1327,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1342,65 +1377,70 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
+          <t>🟢 Ready to Move (2 yrs old • Instant Handover)</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
           <t>Final Units with OC Handover</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>3 BHK Ultra-Luxury</t>
         </is>
       </c>
-      <c r="N8" t="n">
+      <c r="O8" t="n">
         <v>1950</v>
       </c>
-      <c r="O8" t="n">
+      <c r="P8" t="n">
         <v>16200</v>
       </c>
-      <c r="P8" t="n">
+      <c r="Q8" t="n">
         <v>3.16</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="R8" t="n">
         <v>18</v>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>Elevated Geological Ridge (+12m above tidal surge)</t>
         </is>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>MBBR Biological STP</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="V8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr">
+      <c r="W8" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="W8" t="n">
+      <c r="X8" t="n">
         <v>95.09999999999999</v>
       </c>
-      <c r="X8" t="inlineStr">
+      <c r="Y8" t="inlineStr">
         <is>
           <t>✅ Critic AI Validated</t>
         </is>
       </c>
-      <c r="Y8" t="inlineStr">
+      <c r="Z8" t="inlineStr">
         <is>
           <t>https://www.rera.tn.gov.in/</t>
         </is>
       </c>
-      <c r="Z8" t="inlineStr">
+      <c r="AA8" t="inlineStr">
         <is>
           <t>State RERA Registry (Puravankara Limited Legal Filing) | Municipal Stormwater Master Plan (GIS Contour Elevation) | TomTom / Google Mobility Commute Index | Public Works Department / Metro Phase Infrastructure Blueprint</t>
         </is>
@@ -1414,7 +1454,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1464,65 +1504,70 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
+          <t>🏗️ Under Construction (Q3 2026 • 11 mos)</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
           <t>Tower Jade (Structure 14th Floor)</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>3 BHK Corporate Suite</t>
         </is>
       </c>
-      <c r="N9" t="n">
+      <c r="O9" t="n">
         <v>1780</v>
       </c>
-      <c r="O9" t="n">
+      <c r="P9" t="n">
         <v>14500</v>
       </c>
-      <c r="P9" t="n">
+      <c r="Q9" t="n">
         <v>2.58</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="R9" t="n">
         <v>7.5</v>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>High Raised Plinth (+1.8m above OMR road grade)</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>MBBR Biological STP</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
+      <c r="V9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="V9" t="inlineStr">
+      <c r="W9" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="W9" t="n">
+      <c r="X9" t="n">
         <v>93.59999999999999</v>
       </c>
-      <c r="X9" t="inlineStr">
+      <c r="Y9" t="inlineStr">
         <is>
           <t>✅ Critic AI Validated</t>
         </is>
       </c>
-      <c r="Y9" t="inlineStr">
+      <c r="Z9" t="inlineStr">
         <is>
           <t>https://www.rera.tn.gov.in/</t>
         </is>
       </c>
-      <c r="Z9" t="inlineStr">
+      <c r="AA9" t="inlineStr">
         <is>
           <t>State RERA Registry (Brigade Group Legal Filing) | Municipal Stormwater Master Plan (GIS Contour Elevation) | TomTom / Google Mobility Commute Index | Public Works Department / Metro Phase Infrastructure Blueprint</t>
         </is>
@@ -1536,7 +1581,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1586,65 +1631,70 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
+          <t>🏗️ Under Construction (Dec 2026 • 14 mos)</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
           <t>Sky Villas Block C</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>3 BHK Metro Core</t>
         </is>
       </c>
-      <c r="N10" t="n">
+      <c r="O10" t="n">
         <v>1520</v>
       </c>
-      <c r="O10" t="n">
+      <c r="P10" t="n">
         <v>12800</v>
       </c>
-      <c r="P10" t="n">
+      <c r="Q10" t="n">
         <v>1.95</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="R10" t="n">
         <v>15</v>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="S10" t="inlineStr">
         <is>
           <t>Zero Inundation (Natural High Alluvial Ridge)</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>MBBR Biological STP</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="V10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr">
+      <c r="W10" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="W10" t="n">
+      <c r="X10" t="n">
         <v>92.8</v>
       </c>
-      <c r="X10" t="inlineStr">
+      <c r="Y10" t="inlineStr">
         <is>
           <t>✅ Critic AI Validated</t>
         </is>
       </c>
-      <c r="Y10" t="inlineStr">
+      <c r="Z10" t="inlineStr">
         <is>
           <t>https://www.rera.tn.gov.in/</t>
         </is>
       </c>
-      <c r="Z10" t="inlineStr">
+      <c r="AA10" t="inlineStr">
         <is>
           <t>State RERA Registry (Appaswamy Real Estates Legal Filing) | Municipal Stormwater Master Plan (GIS Contour Elevation) | TomTom / Google Mobility Commute Index | Public Works Department / Metro Phase Infrastructure Blueprint</t>
         </is>
@@ -1658,7 +1708,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1708,67 +1758,1088 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
+          <t>🏗️ Near Completion (Q1 2026 • 5 mos)</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
           <t>Tower Aster (Pre-Handover Snagging)</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>3 BHK Luxury</t>
         </is>
       </c>
-      <c r="N11" t="n">
+      <c r="O11" t="n">
         <v>2680</v>
       </c>
-      <c r="O11" t="n">
+      <c r="P11" t="n">
         <v>24500</v>
       </c>
-      <c r="P11" t="n">
+      <c r="Q11" t="n">
         <v>6.57</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="R11" t="n">
         <v>235</v>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="S11" t="inlineStr">
         <is>
           <t>Zero Inundation (Elevated Foothills Slope)</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>MBBR Biological STP</t>
         </is>
       </c>
-      <c r="T11" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="V11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
+      <c r="W11" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="W11" t="n">
+      <c r="X11" t="n">
         <v>97.40000000000001</v>
       </c>
-      <c r="X11" t="inlineStr">
+      <c r="Y11" t="inlineStr">
         <is>
           <t>✅ Critic AI Validated</t>
         </is>
       </c>
-      <c r="Y11" t="inlineStr">
+      <c r="Z11" t="inlineStr">
         <is>
           <t>https://haryanarera.gov.in/</t>
         </is>
       </c>
-      <c r="Z11" t="inlineStr">
+      <c r="AA11" t="inlineStr">
         <is>
           <t>State RERA Registry (DLF Limited Legal Filing) | Municipal Stormwater Master Plan (GIS Contour Elevation) | TomTom / Google Mobility Commute Index | Public Works Department / Metro Phase Infrastructure Blueprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>51c49e4ceb</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Eldeco Live Neoma</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Delhi-NCR</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Sector 150 - Noida Expressway</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Eldeco Group</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Tier 1 Regional Champion (North)</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>94%</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Noida International Airport Jewar (20 mins via Yamuna Exp) + Aqua Line Metro Extension + 80% designated green zone</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>+62.5%</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>🏗️ Under Construction (Dec 2026 • 14 mos)</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Phase 3 Sky Residences</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>3 BHK Sports City</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
+        <v>1750</v>
+      </c>
+      <c r="P12" t="n">
+        <v>10800</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="R12" t="n">
+        <v>204</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>High Engineered Plinth (Outside Yamuna O-Zone)</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>MBBR Biological STP</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X12" t="n">
+        <v>94</v>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>https://up-rera.in/</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>State RERA Registry (Eldeco Group Legal Filing) | Municipal Stormwater Master Plan (GIS Contour Elevation) | TomTom / Google Mobility Commute Index | Public Works Department / Metro Phase Infrastructure Blueprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>a570222d4f</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Godrej South Estate</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Delhi-NCR</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Okhla Phase 1 - South Delhi</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Godrej Properties</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Tier 1 Premier National</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>93%</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Delhi Metro Magenta &amp; Violet Lines intersection + DDA Transit-Oriented Development (TOD) corridor</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>+59.0%</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>March 2027</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>🚀 Upcoming Pre-Launch (March 2027 • ~2 yrs)</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Tower 6 &amp; 7 (Under Construction)</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>3 BHK Ultra Luxury</t>
+        </is>
+      </c>
+      <c r="O13" t="n">
+        <v>2150</v>
+      </c>
+      <c r="P13" t="n">
+        <v>22500</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>4.84</v>
+      </c>
+      <c r="R13" t="n">
+        <v>218</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>Zero Inundation (High Ridge Flank)</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>MBBR Biological STP</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X13" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>https://delhirera.in/</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>State RERA Registry (Godrej Properties Legal Filing) | Municipal Stormwater Master Plan (GIS Contour Elevation) | TomTom / Google Mobility Commute Index | Public Works Department / Metro Phase Infrastructure Blueprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>aeeaad28fd</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>My Home Bhooja</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>HITECH City - Knowledge City</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>My Home Group</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Tier 1 Regional Champion</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>95%</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Hyderabad Metro Blue Line station walking distance + Inorbit Mall flyover + Bio-Diversity flyover network</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>+55.0%</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>Q4 2026</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>🟢 Ready to Move (3 yrs old • Luxury OC)</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Tower Sapphire (Structure Complete)</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>3 BHK Iconic Skyvilla</t>
+        </is>
+      </c>
+      <c r="O14" t="n">
+        <v>2595</v>
+      </c>
+      <c r="P14" t="n">
+        <v>14800</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="R14" t="n">
+        <v>582</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Zero Inundation (High Granite Hillock)</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>MBBR Biological STP</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X14" t="n">
+        <v>96.5</v>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+      <c r="Z14" t="inlineStr">
+        <is>
+          <t>https://rera.telangana.gov.in/</t>
+        </is>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>State RERA Registry (My Home Group Legal Filing) | Municipal Stormwater Master Plan (GIS Contour Elevation) | TomTom / Google Mobility Commute Index | Public Works Department / Metro Phase Infrastructure Blueprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>c8d41993ae</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Aparna Sarovar Zenith</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Nallagandla - Gachibowli</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Aparna Constructions</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Tier 1 Regional Champion</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>92%</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Tellapur-Nallagandla 100ft road to ORR Exit 2 + Citizen Hospital healthcare corridor</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>+41.0%</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>Ready to Move</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>🟢 Ready to Move (5 yrs old • 100% Occupied)</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Occupancy Certificate Issued</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>3 BHK Gated Park</t>
+        </is>
+      </c>
+      <c r="O15" t="n">
+        <v>1850</v>
+      </c>
+      <c r="P15" t="n">
+        <v>9800</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>1.81</v>
+      </c>
+      <c r="R15" t="n">
+        <v>560</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Zero Inundation (High Rocky Ridge)</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>MBBR Biological STP</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W15" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X15" t="n">
+        <v>94.2</v>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+      <c r="Z15" t="inlineStr">
+        <is>
+          <t>https://rera.telangana.gov.in/</t>
+        </is>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>State RERA Registry (Aparna Constructions Legal Filing) | Municipal Stormwater Master Plan (GIS Contour Elevation) | TomTom / Google Mobility Commute Index | Public Works Department / Metro Phase Infrastructure Blueprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2b9b6bd1c6</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Prestige Clairemont</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Kokapet - Neopolis SEZ</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Prestige Group</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Tier 1 Premier National</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>95%</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Kokapet Neopolis SEZ 45m master roads + Direct ORR Trumpet Interchange + 100-acre Commercial CBD</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>+58.0%</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>March 2027</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>🏗️ Under Construction (March 2027 • 17 mos)</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Phase 2 Green Towers</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>3 BHK Premium High-Rise</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>1980</v>
+      </c>
+      <c r="P16" t="n">
+        <v>11500</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>2.28</v>
+      </c>
+      <c r="R16" t="n">
+        <v>578</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Zero Inundation (Natural Granitic Slope)</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>MBBR Biological STP</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W16" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X16" t="n">
+        <v>95.40000000000001</v>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+      <c r="Z16" t="inlineStr">
+        <is>
+          <t>https://rera.telangana.gov.in/</t>
+        </is>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>State RERA Registry (Prestige Group Legal Filing) | Municipal Stormwater Master Plan (GIS Contour Elevation) | TomTom / Google Mobility Commute Index | Public Works Department / Metro Phase Infrastructure Blueprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>17c2320cfe</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Eldeco Surya Greens</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Varanasi &amp; Eastern UP 100km Corridor</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Shivpur - North Varanasi Ridge</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Eldeco Group</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Tier 1 Regional Champion (North)</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>93%</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Varanasi 6-Lane Ring Road Phase 2 + Babatpur Airport 4-Lane Highway + Smart City Multi-Modal Hub</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>+64.0%</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Dec 2026</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>🏗️ Under Construction (Dec 2026 • 14 mos)</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Phase 2 Ganga View Blocks</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>3 BHK Prime Gated</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>1550</v>
+      </c>
+      <c r="P17" t="n">
+        <v>6900</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="R17" t="n">
+        <v>85</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Zero Inundation (High Alluvial Ridge: +11m above Ganga HFL)</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>MBBR Biological STP</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W17" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X17" t="n">
+        <v>94.40000000000001</v>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+      <c r="Z17" t="inlineStr">
+        <is>
+          <t>https://up-rera.in/</t>
+        </is>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>State RERA Registry (Eldeco Group Legal Filing) | Municipal Stormwater Master Plan (GIS Contour Elevation) | TomTom / Google Mobility Commute Index | Public Works Department / Metro Phase Infrastructure Blueprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>209a26b4c1</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Omaxe Heights Prayagraj</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Varanasi &amp; Eastern UP 100km Corridor</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Civil Lines - Prayagraj</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Omaxe Limited</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Tier 1 National Player</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>92%</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Prayagraj Mahakumbh 2025 Infrastructure Works + 6-lane Ganga Expressway link to Meerut/Delhi</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>+46.0%</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Ready to Move</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>🟢 Ready to Move (2 yrs old • Registry Ready)</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Civil Lines Completed Enclave</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>3 BHK Royal Luxury</t>
+        </is>
+      </c>
+      <c r="O18" t="n">
+        <v>1720</v>
+      </c>
+      <c r="P18" t="n">
+        <v>8200</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>1.41</v>
+      </c>
+      <c r="R18" t="n">
+        <v>98</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Zero Inundation (British Grid Elevated Plateau: +14m above Sangam)</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>MBBR Biological STP</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X18" t="n">
+        <v>93.5</v>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>https://up-rera.in/</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>State RERA Registry (Omaxe Limited Legal Filing) | Municipal Stormwater Master Plan (GIS Contour Elevation) | TomTom / Google Mobility Commute Index | Public Works Department / Metro Phase Infrastructure Blueprint</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>e654fae528</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Kashi Royal Greens</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Varanasi &amp; Eastern UP 100km Corridor</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Babatpur - Airport Corridor</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Roma Builders</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Tier 1 Regional Champion (Varanasi)</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>94%</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>LBS International Airport expansion (New Terminal &amp; Cargo Complex) + Varanasi Ring Road Phase 2 interchange</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>+60.5%</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Q2 2027</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>🚀 Upcoming Pre-Launch (Q2 2027 • ~20 mos)</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Highway Meadows Tower 3</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>3 BHK Airport Gated</t>
+        </is>
+      </c>
+      <c r="O19" t="n">
+        <v>1480</v>
+      </c>
+      <c r="P19" t="n">
+        <v>5800</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="R19" t="n">
+        <v>89</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>Zero Inundation (High Continental Plateau)</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>MBBR Biological STP</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="X19" t="n">
+        <v>93.09999999999999</v>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>https://up-rera.in/</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>State RERA Registry (Roma Builders Legal Filing) | Municipal Stormwater Master Plan (GIS Contour Elevation) | TomTom / Google Mobility Commute Index | Public Works Department / Metro Phase Infrastructure Blueprint</t>
         </is>
       </c>
     </row>
@@ -1783,7 +2854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T11"/>
+  <dimension ref="A1:U19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1839,50 +2910,55 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
+          <t>Plot Status &amp; Handover</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>Plot Sizes (sqft)</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Price / Sqft (INR)</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Starting Ticket</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Elevation (m MSL)</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Statutory Authority</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Soil Percolation</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Flood Exposure</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>Appreciation Score</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>Critic AI Status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>Approval Registry Link</t>
         </is>
@@ -1896,7 +2972,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1941,44 +3017,49 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
+          <t>🟢 Ready for Immediate Registry &amp; Villa Construction</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
           <t>1,500 - 4,000 sqft</t>
         </is>
       </c>
-      <c r="L2" t="n">
+      <c r="M2" t="n">
         <v>8900</v>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>₹133.5 Lakhs - ₹356.0 Lakhs</t>
         </is>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>896</v>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>BMRDA &amp; RERA Approved (PRM/KA/RERA/1251/308/PR/210824/004289)</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>Red Sandy Loam (Rapid natural percolation, zero water stagnation)</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>Zero Inundation (High Ridge Saddle)</t>
         </is>
       </c>
-      <c r="R2" t="n">
+      <c r="S2" t="n">
         <v>95.8</v>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>✅ Critic AI Validated</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>https://rera.karnataka.gov.in/</t>
         </is>
@@ -1992,7 +3073,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -2037,44 +3118,49 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
+          <t>🟢 Ready for Immediate Registry &amp; Villa Construction</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
           <t>1,200 - 3,200 sqft</t>
         </is>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>6400</v>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>₹76.8 Lakhs - ₹204.8 Lakhs</t>
         </is>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>925</v>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>BIAAPA &amp; RERA Approved</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
+      <c r="Q3" t="inlineStr">
         <is>
           <t>Alluvial gravely loam, zero water retention</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>Zero Inundation (High Continental Divide)</t>
         </is>
       </c>
-      <c r="R3" t="n">
+      <c r="S3" t="n">
         <v>94.5</v>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="T3" t="inlineStr">
         <is>
           <t>✅ Critic AI Validated</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>https://rera.karnataka.gov.in/</t>
         </is>
@@ -2088,7 +3174,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2133,44 +3219,49 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
+          <t>🟢 Ready for Immediate Registry &amp; Villa Construction</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
           <t>1,800 - 3,500 sqft</t>
         </is>
       </c>
-      <c r="L4" t="n">
+      <c r="M4" t="n">
         <v>7800</v>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>₹140.4 Lakhs - ₹273.0 Lakhs</t>
         </is>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>918</v>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>BIAAPA Approved &amp; Karnataka RERA Registered</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Permeable red murrum, naturally self-draining</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>Zero Inundation (Natural Granitic Plateau)</t>
         </is>
       </c>
-      <c r="R4" t="n">
+      <c r="S4" t="n">
         <v>94.2</v>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>✅ Critic AI Validated</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>https://rera.karnataka.gov.in/</t>
         </is>
@@ -2184,7 +3275,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2229,44 +3320,49 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
+          <t>🏗️ Under Development (Phased Handover Q4 2025)</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
           <t>1,800 - 4,500 sqft</t>
         </is>
       </c>
-      <c r="L5" t="n">
+      <c r="M5" t="n">
         <v>9200</v>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>₹165.6 Lakhs - ₹414.0 Lakhs</t>
         </is>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>35</v>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>CIDCO / NA Permission / MahaRERA Approved</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
+      <c r="Q5" t="inlineStr">
         <is>
           <t>Basaltic murrum with fast gravitational runoff to Prabalmachi stream</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>Zero Inundation (Elevated Foothills Plateau)</t>
         </is>
       </c>
-      <c r="R5" t="n">
+      <c r="S5" t="n">
         <v>95.40000000000001</v>
       </c>
-      <c r="S5" t="inlineStr">
+      <c r="T5" t="inlineStr">
         <is>
           <t>✅ Critic AI Validated</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>https://maharera.mahaonline.gov.in/</t>
         </is>
@@ -2280,7 +3376,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -2325,44 +3421,49 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
+          <t>🟢 Ready for Immediate Registry &amp; Villa Construction</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
           <t>1,500 - 3,500 sqft</t>
         </is>
       </c>
-      <c r="L6" t="n">
+      <c r="M6" t="n">
         <v>4800</v>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>₹72.0 Lakhs - ₹168.0 Lakhs</t>
         </is>
       </c>
-      <c r="N6" t="n">
+      <c r="O6" t="n">
         <v>62</v>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>MahaRERA &amp; Town Planning Sanctioned</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>Laterite hilly gravel with instantaneous runoff</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>Zero Inundation (Mountain Ridge)</t>
         </is>
       </c>
-      <c r="R6" t="n">
+      <c r="S6" t="n">
         <v>93</v>
       </c>
-      <c r="S6" t="inlineStr">
+      <c r="T6" t="inlineStr">
         <is>
           <t>✅ Critic AI Validated</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>https://maharera.mahaonline.gov.in/</t>
         </is>
@@ -2376,7 +3477,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -2421,44 +3522,49 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
+          <t>🟢 Ready for Immediate Registry &amp; Villa Construction</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
           <t>1,200 - 2,500 sqft</t>
         </is>
       </c>
-      <c r="L7" t="n">
+      <c r="M7" t="n">
         <v>6500</v>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>₹78.0 Lakhs - ₹162.5 Lakhs</t>
         </is>
       </c>
-      <c r="N7" t="n">
+      <c r="O7" t="n">
         <v>24</v>
       </c>
-      <c r="O7" t="inlineStr">
+      <c r="P7" t="inlineStr">
         <is>
           <t>MahaRERA Registered &amp; KDMC Sanctioned</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
+      <c r="Q7" t="inlineStr">
         <is>
           <t>Hard murrum plateau, engineered stormwater retention lake</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t>Zero Inundation (Engineered Township Tableland)</t>
         </is>
       </c>
-      <c r="R7" t="n">
+      <c r="S7" t="n">
         <v>93.59999999999999</v>
       </c>
-      <c r="S7" t="inlineStr">
+      <c r="T7" t="inlineStr">
         <is>
           <t>✅ Critic AI Validated</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>https://maharera.mahaonline.gov.in/</t>
         </is>
@@ -2472,7 +3578,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -2517,44 +3623,49 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
+          <t>🟢 Ready for Immediate Registry &amp; Villa Construction</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
           <t>1,200 - 3,000 sqft</t>
         </is>
       </c>
-      <c r="L8" t="n">
+      <c r="M8" t="n">
         <v>7500</v>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>₹90.0 Lakhs - ₹225.0 Lakhs</t>
         </is>
       </c>
-      <c r="N8" t="n">
+      <c r="O8" t="n">
         <v>14</v>
       </c>
-      <c r="O8" t="inlineStr">
+      <c r="P8" t="inlineStr">
         <is>
           <t>CMDA &amp; TNRERA Approved</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
+      <c r="Q8" t="inlineStr">
         <is>
           <t>Sandy loam with immediate absorption</t>
         </is>
       </c>
-      <c r="Q8" t="inlineStr">
+      <c r="R8" t="inlineStr">
         <is>
           <t>Zero Inundation (High Natural Dune Ridge: +4.5m above marshland datum)</t>
         </is>
       </c>
-      <c r="R8" t="n">
+      <c r="S8" t="n">
         <v>94</v>
       </c>
-      <c r="S8" t="inlineStr">
+      <c r="T8" t="inlineStr">
         <is>
           <t>✅ Critic AI Validated</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>https://www.rera.tn.gov.in/</t>
         </is>
@@ -2568,7 +3679,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -2613,44 +3724,49 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
+          <t>🏗️ Under Development (Q3 2025 Handover)</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
           <t>1,200 - 2,400 sqft</t>
         </is>
       </c>
-      <c r="L9" t="n">
+      <c r="M9" t="n">
         <v>4800</v>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>₹57.6 Lakhs - ₹115.2 Lakhs</t>
         </is>
       </c>
-      <c r="N9" t="n">
+      <c r="O9" t="n">
         <v>22</v>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="P9" t="inlineStr">
         <is>
           <t>CMDA Approved &amp; TNRERA Registered</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="Q9" t="inlineStr">
         <is>
           <t>Red gravely clay loam, good drainage</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="R9" t="inlineStr">
         <is>
           <t>Zero Inundation (High GST Ridge)</t>
         </is>
       </c>
-      <c r="R9" t="n">
+      <c r="S9" t="n">
         <v>92.2</v>
       </c>
-      <c r="S9" t="inlineStr">
+      <c r="T9" t="inlineStr">
         <is>
           <t>✅ Critic AI Validated</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>https://www.rera.tn.gov.in/</t>
         </is>
@@ -2664,7 +3780,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2709,44 +3825,49 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
+          <t>🟢 Ready for Immediate Registry &amp; Villa Construction</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
           <t>1,200 - 3,200 sqft</t>
         </is>
       </c>
-      <c r="L10" t="n">
+      <c r="M10" t="n">
         <v>4200</v>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>₹50.4 Lakhs - ₹134.4 Lakhs</t>
         </is>
       </c>
-      <c r="N10" t="n">
+      <c r="O10" t="n">
         <v>28</v>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>CMDA Sanctioned &amp; TNRERA Approved</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>Coarse sandy gravel, rapid infiltration</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr">
+      <c r="R10" t="inlineStr">
         <is>
           <t>Zero Inundation (High Interfluvial Ridge)</t>
         </is>
       </c>
-      <c r="R10" t="n">
+      <c r="S10" t="n">
         <v>92.8</v>
       </c>
-      <c r="S10" t="inlineStr">
+      <c r="T10" t="inlineStr">
         <is>
           <t>✅ Critic AI Validated</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>https://www.rera.tn.gov.in/</t>
         </is>
@@ -2760,7 +3881,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2805,46 +3926,859 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
+          <t>🟢 Ready for Immediate Registry &amp; Villa Construction</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
           <t>4,050 - 9,000 sqft (450 - 1000 sq yd)</t>
         </is>
       </c>
-      <c r="L11" t="n">
+      <c r="M11" t="n">
         <v>19500</v>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>₹789.7 Lakhs - ₹1,755.0 Lakhs</t>
         </is>
       </c>
-      <c r="N11" t="n">
+      <c r="O11" t="n">
         <v>232</v>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="P11" t="inlineStr">
         <is>
           <t>DTCP Haryana Licenced Colony &amp; HARERA Registered</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
+      <c r="Q11" t="inlineStr">
         <is>
           <t>Semi-arid sandy loam, rapid storm absorption</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
+      <c r="R11" t="inlineStr">
         <is>
           <t>Zero Inundation (High Natural Interfluvial Ridge)</t>
         </is>
       </c>
-      <c r="R11" t="n">
+      <c r="S11" t="n">
         <v>96.8</v>
       </c>
-      <c r="S11" t="inlineStr">
+      <c r="T11" t="inlineStr">
         <is>
           <t>✅ Critic AI Validated</t>
         </is>
       </c>
-      <c r="T11" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>https://haryanarera.gov.in/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>8d0b5e2194</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Signature Global Park Plots</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Delhi-NCR</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Sector 36 Sohna - South of Gurugram</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Signature Global</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>93%</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Sohna Elevated Expressway (15 mins to Subhash Chowk) + Delhi-Mumbai Expressway starting interchange</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>+60.0%</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Immediate Registration &amp; Possession</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>🟢 Ready for Immediate Registry &amp; Villa Construction</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>1,080 - 2,250 sqft</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
+        <v>8200</v>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>₹88.5 Lakhs - ₹184.5 Lakhs</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
+        <v>248</v>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>DTCP Deen Dayal Jan Awas Yojna (DDJAY) &amp; HARERA</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Aravali foothill gravel, high natural runoff</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>Zero Inundation (Elevated Foothill Gradient)</t>
+        </is>
+      </c>
+      <c r="S12" t="n">
+        <v>94</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>https://haryanarera.gov.in/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>19996fe844</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Godrej Palm Retreat Plotted Enclave</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Delhi-NCR</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Sector 150 - Noida Expressway</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Godrej Properties</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>95%</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Direct expressway link to Noida International Airport Jewar + Multi-modal transit hub</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>+65.0%</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Ready for Construction</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>🟢 Ready for Immediate Registry &amp; Villa Construction</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>1,800 - 4,500 sqft</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>14200</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>₹255.6 Lakhs - ₹639.0 Lakhs</t>
+        </is>
+      </c>
+      <c r="O13" t="n">
+        <v>205</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Noida Authority Sanctioned &amp; UP RERA Registered</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Engineered sand gravel bed with rapid drainage fall</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>Zero Inundation (High Engineered Plinth)</t>
+        </is>
+      </c>
+      <c r="S13" t="n">
+        <v>95</v>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>https://up-rera.in/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>dabc1e95d2</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>My Home Ankura Plotted Enclave</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Tellapur - Financial District Extn</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>My Home Group</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>96%</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Hyderabad Radial Road 7 expansion + Tellapur to Kokapet Trumpet Interchange + Multi-Modal MMTS Tellapur station</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>+75.0%</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Ready for Construction</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>🟢 Ready for Immediate Registry &amp; Villa Construction</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2,400 - 4,800 sqft</t>
+        </is>
+      </c>
+      <c r="M14" t="n">
+        <v>9800</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>₹235.2 Lakhs - ₹470.4 Lakhs</t>
+        </is>
+      </c>
+      <c r="O14" t="n">
+        <v>574</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>HMDA &amp; TSRERA Registered</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Granite weathered red soil (High percolation gradient)</t>
+        </is>
+      </c>
+      <c r="R14" t="inlineStr">
+        <is>
+          <t>Zero Inundation (High Granitic Ridge)</t>
+        </is>
+      </c>
+      <c r="S14" t="n">
+        <v>95.59999999999999</v>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>https://rera.telangana.gov.in/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>feadbd3236</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Aparna Dharti Gated Plots</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Dundigal - ORR Exit 5</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Aparna Constructions</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>92%</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Hyderabad Regional Ring Road (RRR) northern quadrant + Medchal pharmaceutical logistics hub</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>+80.0%</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Immediate Villa Handover</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>🟢 Ready for Immediate Registry &amp; Villa Construction</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>1,800 - 3,600 sqft</t>
+        </is>
+      </c>
+      <c r="M15" t="n">
+        <v>5200</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>₹93.6 Lakhs - ₹187.2 Lakhs</t>
+        </is>
+      </c>
+      <c r="O15" t="n">
+        <v>598</v>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>HMDA &amp; TSRERA Registered</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Red gravel soil, zero water accumulation</t>
+        </is>
+      </c>
+      <c r="R15" t="inlineStr">
+        <is>
+          <t>Zero Inundation (Highest Elevation Plateau in Hyderabad: 598m)</t>
+        </is>
+      </c>
+      <c r="S15" t="n">
+        <v>93.2</v>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>https://rera.telangana.gov.in/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>e7446458ac</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Rajapushpa Green Dale Plots</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Tellapur - Osmansagar Ridge</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Rajapushpa Properties</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>95%</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Neopolis 100ft arterial link + Gopanpally flyover to Financial District</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>+65.0%</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Ready for Construction</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>🟢 Ready for Immediate Registry &amp; Villa Construction</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2,700 - 5,400 sqft</t>
+        </is>
+      </c>
+      <c r="M16" t="n">
+        <v>10500</v>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>₹283.5 Lakhs - ₹567.0 Lakhs</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>568</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>HMDA Approved Layout &amp; TSRERA</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Rocky basaltic terrain, zero water retention</t>
+        </is>
+      </c>
+      <c r="R16" t="inlineStr">
+        <is>
+          <t>Zero Inundation (High Continental Divide Ridge)</t>
+        </is>
+      </c>
+      <c r="S16" t="n">
+        <v>95</v>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>https://rera.telangana.gov.in/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>cefb99f217</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Eldeco Shaurya Gated Plots</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Varanasi &amp; Eastern UP 100km Corridor</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Varanasi-Lucknow NH-56 Highway, Shivpur Extn</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Eldeco Group</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>94%</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Varanasi Ring Road Phase 2 + Babatpur Airport Aero-City Logistic Zone + Kashi Integrated Smart Transit Hub</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>+85.0%</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Immediate Registration</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>🟢 Ready for Immediate Registry &amp; Villa Construction</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>1,350 - 3,600 sqft (150 - 400 sq yd)</t>
+        </is>
+      </c>
+      <c r="M17" t="n">
+        <v>4500</v>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>₹60.7 Lakhs - ₹162.0 Lakhs</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>88</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>VDA (Varanasi Development Authority) Sanctioned &amp; UP RERA Registered</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>High coarse silt-loam terrace (Immune to Ganga &amp; Varuna backwaters: +14m above Ganga 1978 HFL)</t>
+        </is>
+      </c>
+      <c r="R17" t="inlineStr">
+        <is>
+          <t>Zero Inundation (Immune High Terrace: 88m MSL vs Ganga HFL 73.9m)</t>
+        </is>
+      </c>
+      <c r="S17" t="n">
+        <v>94.59999999999999</v>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>https://up-rera.in/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>398bfa7909</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>PDA Sangam Vihar Gated Plotted Scheme</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Varanasi &amp; Eastern UP 100km Corridor</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Civil Lines Extn - Jhalwa Elevated Sector, Prayagraj</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Prayagraj Development Authority (PDA)</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>93%</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Prayagraj Mahakumbh 2025 Transit Grid + IIIT Prayagraj Knowledge Park + Direct Ganga Expressway Ramp</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>+90.0%</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Ready for Registry</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>🟢 Ready for Immediate Registry &amp; Villa Construction</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>1,800 - 4,500 sqft (200 - 500 sq yd)</t>
+        </is>
+      </c>
+      <c r="M18" t="n">
+        <v>4800</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>₹86.4 Lakhs - ₹216.0 Lakhs</t>
+        </is>
+      </c>
+      <c r="O18" t="n">
+        <v>102</v>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>PDA Statutory Government Scheme &amp; Freehold Registry</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Consolidated alluvial ridge, natural gravity stormwater fall into Sasur Khaderi ravine</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>Zero Inundation (High Alluvial Ridge: 102m MSL vs Sangam HFL 84.7m)</t>
+        </is>
+      </c>
+      <c r="S18" t="n">
+        <v>93.8</v>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>https://up-rera.in/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>684503c863</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Mirzapur Vindhya Enclave Gated Plots</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Varanasi &amp; Eastern UP 100km Corridor</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Vindhyachal Corridor Highway NH-135, Mirzapur</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Roma Builders &amp; Promoters</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>92%</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>Maa Vindhyavasini Temple Corridor Pilgrimage Redevelopment + Dedicated 4-lane Ring Highway to Varanasi</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>+65.0%</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Ready for Construction</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>🟢 Ready for Immediate Registry &amp; Villa Construction</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>1,500 - 3,000 sqft</t>
+        </is>
+      </c>
+      <c r="M19" t="n">
+        <v>3200</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>₹48.0 Lakhs - ₹96.0 Lakhs</t>
+        </is>
+      </c>
+      <c r="O19" t="n">
+        <v>94</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>VDA &amp; UP RERA Registered</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Sandstone rocky base with fast surface gradient to natural hill ravines</t>
+        </is>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>Zero Inundation (High Vindhyan Foothill Ridge)</t>
+        </is>
+      </c>
+      <c r="S19" t="n">
+        <v>92.5</v>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>https://up-rera.in/</t>
         </is>
       </c>
     </row>
@@ -2859,7 +4793,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2952,7 +4886,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -3020,7 +4954,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -3088,7 +5022,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -3156,7 +5090,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -3224,7 +5158,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -3292,7 +5226,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -3360,7 +5294,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -3428,7 +5362,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -3496,7 +5430,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -3564,7 +5498,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -3619,6 +5553,550 @@
         </is>
       </c>
       <c r="P11" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>9388152d2c</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Godrej Woods</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Delhi-NCR</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Sector 43 - Central Noida</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Godrej Properties</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>3 BHK Forest Theme (1850 sqft)</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>72000</v>
+      </c>
+      <c r="I12" t="n">
+        <v>6800</v>
+      </c>
+      <c r="J12" t="n">
+        <v>180000</v>
+      </c>
+      <c r="K12" t="n">
+        <v>3.84</v>
+      </c>
+      <c r="L12" t="n">
+        <v>2</v>
+      </c>
+      <c r="M12" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="N12" t="n">
+        <v>94.2</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>94%</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>e6187aa395</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Mahagun Moderne</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Delhi-NCR</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Sector 78 - Central Noida</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Mahagun Group</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>3 BHK Premium Gated (1550 sqft)</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>48000</v>
+      </c>
+      <c r="I13" t="n">
+        <v>4500</v>
+      </c>
+      <c r="J13" t="n">
+        <v>100000</v>
+      </c>
+      <c r="K13" t="n">
+        <v>3.97</v>
+      </c>
+      <c r="L13" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="M13" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="N13" t="n">
+        <v>93</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>91%</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>4d1d3d4d3e</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Aparna Serene Park</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Gachibowli - Kondapur</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Aparna Constructions</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>3 BHK Gated High-Rise (1710 sqft)</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>62000</v>
+      </c>
+      <c r="I14" t="n">
+        <v>5500</v>
+      </c>
+      <c r="J14" t="n">
+        <v>150000</v>
+      </c>
+      <c r="K14" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="L14" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="M14" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="N14" t="n">
+        <v>95</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>94%</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>aaed5f5e77</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Rajapushpa Provincia</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Narsingi - Financial District</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Rajapushpa Properties</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>3 BHK Ultra-Luxury (2020 sqft)</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>68000</v>
+      </c>
+      <c r="I15" t="n">
+        <v>6000</v>
+      </c>
+      <c r="J15" t="n">
+        <v>180000</v>
+      </c>
+      <c r="K15" t="n">
+        <v>3.98</v>
+      </c>
+      <c r="L15" t="n">
+        <v>3</v>
+      </c>
+      <c r="M15" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="N15" t="n">
+        <v>94.09999999999999</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>95%</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>b500a57a96</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>My Home Avatar</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Hyderabad</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Puppalaguda - Financial District</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>My Home Group</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>3 BHK Master Township (1834 sqft)</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>64000</v>
+      </c>
+      <c r="I16" t="n">
+        <v>5800</v>
+      </c>
+      <c r="J16" t="n">
+        <v>160000</v>
+      </c>
+      <c r="K16" t="n">
+        <v>4.04</v>
+      </c>
+      <c r="L16" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="M16" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="N16" t="n">
+        <v>94.40000000000001</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>94%</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>680de3c27f</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Eldeco Anandam Residency</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Varanasi &amp; Eastern UP 100km Corridor</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Civil Lines - Prayagraj</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Eldeco Group</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>3 BHK Executive (1450 sqft)</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>34000</v>
+      </c>
+      <c r="I17" t="n">
+        <v>3800</v>
+      </c>
+      <c r="J17" t="n">
+        <v>70000</v>
+      </c>
+      <c r="K17" t="n">
+        <v>4.16</v>
+      </c>
+      <c r="L17" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="M17" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N17" t="n">
+        <v>93</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>91%</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>f69fd40a90</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Kashi Smart City Towers</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Varanasi &amp; Eastern UP 100km Corridor</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Shivpur - Cantt Varanasi</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Kashi Infra Developers</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>3 BHK Premium Gated (1400 sqft)</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>28000</v>
+      </c>
+      <c r="I18" t="n">
+        <v>3200</v>
+      </c>
+      <c r="J18" t="n">
+        <v>60000</v>
+      </c>
+      <c r="K18" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="L18" t="n">
+        <v>3</v>
+      </c>
+      <c r="M18" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="N18" t="n">
+        <v>92.40000000000001</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>92%</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>✅ Critic AI Validated</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1e72021816</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-10-03 11:31:17</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Sangam Vihar Residency</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Varanasi &amp; Eastern UP 100km Corridor</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Jhalwa - IT Park Prayagraj</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Omaxe Limited</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>3 BHK Academic Suite (1380 sqft)</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>25000</v>
+      </c>
+      <c r="I19" t="n">
+        <v>2800</v>
+      </c>
+      <c r="J19" t="n">
+        <v>50000</v>
+      </c>
+      <c r="K19" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="L19" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="N19" t="n">
+        <v>92</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>90%</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr">
         <is>
           <t>✅ Critic AI Validated</t>
         </is>
@@ -3688,7 +6166,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3729,7 +6207,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3770,7 +6248,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3811,7 +6289,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3852,7 +6330,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3893,7 +6371,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -3934,7 +6412,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3975,7 +6453,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -4042,7 +6520,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-03 11:23:15</t>
+          <t>2026-10-03 11:31:17</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">

</xml_diff>